<commit_message>
Exploratory of Chen and al. dataset from 2010 to 2022
</commit_message>
<xml_diff>
--- a/BDD.xlsx
+++ b/BDD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\solar-data-china\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E767DF-1232-4D74-A522-C4C179B0A226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8D78C5-AECA-488B-90B8-65D13D2CD123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>

</xml_diff>